<commit_message>
Update Global Branding and CMS config
</commit_message>
<xml_diff>
--- a/public/config.xlsx
+++ b/public/config.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -409,103 +409,135 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>HeroHeading</v>
+        <v>CompanyName</v>
       </c>
       <c r="B2" t="str">
-        <v>Engineering Scalable Digital Systems</v>
+        <v>TechInnoSphere</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>HeroSubheading</v>
+        <v>CompanyLogo</v>
       </c>
       <c r="B3" t="str">
-        <v>TechInnoSphere delivers premium Web Development, AI Solutions, Security Testing, and Enterprise Software.</v>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>HeroButtonPrimaryText</v>
+        <v>Favicon</v>
       </c>
       <c r="B4" t="str">
-        <v>Start Your Project</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>HeroButtonPrimaryLink</v>
+        <v>WhatsAppNumber</v>
       </c>
       <c r="B5" t="str">
-        <v>/contact</v>
+        <v>+917710031550</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>HeroButtonSecondaryText</v>
+        <v>InstagramURL</v>
       </c>
       <c r="B6" t="str">
-        <v>View Our Work</v>
+        <v>https://www.instagram.com/techinnosphere/</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>HeroButtonSecondaryLink</v>
+        <v>FacebookURL</v>
       </c>
       <c r="B7" t="str">
-        <v>/work</v>
+        <v>https://www.facebook.com/profile.php?id=61584937588072</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ContactEmail</v>
+        <v>CompanyAddress</v>
       </c>
       <c r="B8" t="str">
-        <v>contact@techinnosphere.com</v>
+        <v>Mumbai, Maharashtra, India</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ContactPhone</v>
+        <v>ContactEmail</v>
       </c>
       <c r="B9" t="str">
-        <v>+91 9999999999</v>
+        <v>careers@techinnosphere.com</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ContactAddress</v>
+        <v>FooterContent</v>
       </c>
       <c r="B10" t="str">
-        <v>Mumbai, Maharashtra, India</v>
+        <v>© TechInnoSphere. All Rights Reserved.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>LinkedInURL</v>
+        <v>HeroHeading</v>
       </c>
       <c r="B11" t="str">
-        <v>https://linkedin.com</v>
+        <v>Engineering Scalable Digital Systems</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>TwitterURL</v>
+        <v>HeroSubheading</v>
       </c>
       <c r="B12" t="str">
-        <v>https://twitter.com</v>
+        <v>TechInnoSphere delivers premium Web Development, AI Solutions, Security Testing, and Enterprise Software.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
+        <v>HeroButtonPrimaryText</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Start Your Project</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>HeroButtonPrimaryLink</v>
+      </c>
+      <c r="B14" t="str">
+        <v>/contact</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>HeroButtonSecondaryText</v>
+      </c>
+      <c r="B15" t="str">
+        <v>View Our Work</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>HeroButtonSecondaryLink</v>
+      </c>
+      <c r="B16" t="str">
+        <v>/work</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
         <v>CompanyTagline</v>
       </c>
-      <c r="B13" t="str">
+      <c r="B17" t="str">
         <v>From Vision To Software We Build It All.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Integrate official TechInnoSphere logo across the website
</commit_message>
<xml_diff>
--- a/public/config.xlsx
+++ b/public/config.xlsx
@@ -420,7 +420,7 @@
         <v>CompanyLogo</v>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>logo.png</v>
       </c>
     </row>
     <row r="4">
@@ -428,7 +428,7 @@
         <v>Favicon</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>logo.png</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Update generate_dummy_data config and services excel sheets
</commit_message>
<xml_diff>
--- a/public/config.xlsx
+++ b/public/config.xlsx
@@ -1,41 +1,128 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\For Other\fehed\Tech\TechInnoSphere-Single\TechInnoSphere\public\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D932A0-69B9-4C42-B31A-A45EA13727F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>CompanyName</t>
+  </si>
+  <si>
+    <t>TechInnoSphere</t>
+  </si>
+  <si>
+    <t>CompanyLogo</t>
+  </si>
+  <si>
+    <t>logo.png</t>
+  </si>
+  <si>
+    <t>Favicon</t>
+  </si>
+  <si>
+    <t>WhatsAppNumber</t>
+  </si>
+  <si>
+    <t>+917710031550</t>
+  </si>
+  <si>
+    <t>InstagramURL</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/techinnosphere/</t>
+  </si>
+  <si>
+    <t>FacebookURL</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/profile.php?id=61584937588072</t>
+  </si>
+  <si>
+    <t>CompanyAddress</t>
+  </si>
+  <si>
+    <t>Mumbai, Maharashtra, India</t>
+  </si>
+  <si>
+    <t>ContactEmail</t>
+  </si>
+  <si>
+    <t>careers@techinnosphere.com</t>
+  </si>
+  <si>
+    <t>FooterContent</t>
+  </si>
+  <si>
+    <t>© TechInnoSphere. All Rights Reserved.</t>
+  </si>
+  <si>
+    <t>HeroHeading</t>
+  </si>
+  <si>
+    <t>Engineering Scalable Digital Systems</t>
+  </si>
+  <si>
+    <t>HeroSubheading</t>
+  </si>
+  <si>
+    <t>HeroButtonPrimaryText</t>
+  </si>
+  <si>
+    <t>Start Your Project</t>
+  </si>
+  <si>
+    <t>HeroButtonPrimaryLink</t>
+  </si>
+  <si>
+    <t>/contact</t>
+  </si>
+  <si>
+    <t>HeroButtonSecondaryText</t>
+  </si>
+  <si>
+    <t>View Our Work</t>
+  </si>
+  <si>
+    <t>HeroButtonSecondaryLink</t>
+  </si>
+  <si>
+    <t>/work</t>
+  </si>
+  <si>
+    <t>CompanyTagline</t>
+  </si>
+  <si>
+    <t>From Vision To Software We Build It All.</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,13 +152,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,148 +491,154 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="94.3984375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Key</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Value</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>CompanyName</v>
-      </c>
-      <c r="B2" t="str">
-        <v>TechInnoSphere</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>CompanyLogo</v>
-      </c>
-      <c r="B3" t="str">
-        <v>logo.png</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Favicon</v>
-      </c>
-      <c r="B4" t="str">
-        <v>logo.png</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>WhatsAppNumber</v>
-      </c>
-      <c r="B5" t="str">
-        <v>+917710031550</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>InstagramURL</v>
-      </c>
-      <c r="B6" t="str">
-        <v>https://www.instagram.com/techinnosphere/</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>FacebookURL</v>
-      </c>
-      <c r="B7" t="str">
-        <v>https://www.facebook.com/profile.php?id=61584937588072</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>CompanyAddress</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Mumbai, Maharashtra, India</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>ContactEmail</v>
-      </c>
-      <c r="B9" t="str">
-        <v>careers@techinnosphere.com</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>FooterContent</v>
-      </c>
-      <c r="B10" t="str">
-        <v>© TechInnoSphere. All Rights Reserved.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>HeroHeading</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Engineering Scalable Digital Systems</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>HeroSubheading</v>
-      </c>
-      <c r="B12" t="str">
-        <v>TechInnoSphere delivers premium Web Development, AI Solutions, Security Testing, and Enterprise Software.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>HeroButtonPrimaryText</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Start Your Project</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>HeroButtonPrimaryLink</v>
-      </c>
-      <c r="B14" t="str">
-        <v>/contact</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>HeroButtonSecondaryText</v>
-      </c>
-      <c r="B15" t="str">
-        <v>View Our Work</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>HeroButtonSecondaryLink</v>
-      </c>
-      <c r="B16" t="str">
-        <v>/work</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>CompanyTagline</v>
-      </c>
-      <c r="B17" t="str">
-        <v>From Vision To Software We Build It All.</v>
+    <row r="1" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B17"/>
+    <ignoredError sqref="A1:B11 A13:B17 A12" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>